<commit_message>
new versions final and final_low_money
</commit_message>
<xml_diff>
--- a/Versionen/Neg_SP_Einkommen_Strom_v2/game_data.xlsx
+++ b/Versionen/Neg_SP_Einkommen_Strom_v2/game_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\_Privat\Coding\KlimSta\Versionen\Neg_SP_Einkommen_Strom_v2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schneids\code\KlimSta-Brettspiel\Versionen\Neg_SP_Einkommen_Strom_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B7F0F81-1339-41DE-9A7B-9791336EBE3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{622C52E2-77D7-4234-9C8B-ECD51B2D860E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="721" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12660" yWindow="-17484" windowWidth="30936" windowHeight="16776" tabRatio="721" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Massnahmenkarten Spielwerte" sheetId="1" r:id="rId1"/>
@@ -73,9 +73,9 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0" xr:uid="{884F3275-8B47-4A24-9A63-26455AFB7D59}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
     KgCO2/m²a</t>
       </text>
     </comment>
@@ -92,18 +92,18 @@
   <commentList>
     <comment ref="C2" authorId="0" shapeId="0" xr:uid="{EF592111-A8C2-4853-9B03-5FD652A65E13}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t xml:space="preserve">[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
     €/m²
 </t>
       </text>
     </comment>
     <comment ref="H2" authorId="1" shapeId="0" xr:uid="{42E090DF-C6E0-4ACF-94D0-539FD66BF793}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
     Geld token</t>
       </text>
     </comment>
@@ -2193,7 +2193,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="80">
     <dxf>
@@ -2203,6 +2203,151 @@
           <bgColor rgb="FFB7E1CD"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -2696,151 +2841,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF6F8F9"/>
@@ -3240,16 +3240,16 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Heizsystem"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Kosten"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="BauEmissionen"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="SofortCO2" dataDxfId="36">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="SofortCO2" dataDxfId="47">
       <calculatedColumnFormula>Table1[[#This Row],[REAL Sofort CO2]]/kgemission_per_sp</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Strombedarf" dataDxfId="35">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Strombedarf" dataDxfId="46">
       <calculatedColumnFormula>Table1[[#This Row],[REAL Strombedarf]]/real_zu_spiel_strombedarf</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Stromproduktion" dataDxfId="34">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Stromproduktion" dataDxfId="45">
       <calculatedColumnFormula>Table1[[#This Row],[REAL Stromproduktion]]/real_zu_spiel_stromproduktion</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Stromspeicher" dataDxfId="33">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Stromspeicher" dataDxfId="44">
       <calculatedColumnFormula>Table1[[#This Row],[REAL Stromspeicher]]/real_zu_spiel_stromspeicher</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Wärmeschutz"/>
@@ -3257,8 +3257,8 @@
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Zufriedenheit"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="SofortBudget"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="REAL Kosten"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="REAL BauEmissionen" dataDxfId="32"/>
-    <tableColumn id="25" xr3:uid="{8B6CFA43-B9CB-4808-B66A-C728842AC947}" name="REAL Sofort CO2" dataDxfId="31"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="REAL BauEmissionen" dataDxfId="43"/>
+    <tableColumn id="25" xr3:uid="{8B6CFA43-B9CB-4808-B66A-C728842AC947}" name="REAL Sofort CO2" dataDxfId="42"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="REAL Strombedarf"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="REAL Stromproduktion"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="REAL Stromspeicher"/>
@@ -3267,7 +3267,7 @@
     <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Voraussetzung Spalte"/>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Voraussetzung Wert"/>
     <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Voraussetzung Wert NICHT"/>
-    <tableColumn id="26" xr3:uid="{FDB4847F-B10D-4845-B90B-E9D5F945F1B7}" name="EffektParsed" dataDxfId="30">
+    <tableColumn id="26" xr3:uid="{FDB4847F-B10D-4845-B90B-E9D5F945F1B7}" name="EffektParsed" dataDxfId="41">
       <calculatedColumnFormula>_xlfn.TEXTJOIN(
 "XX",
 TRUE,
@@ -3281,7 +3281,7 @@
 IF(D2="FW","XXFW",IF(D2="BIO","XXBI",IF(D2="ABWWP","XXWP",IF(D2="WP","XXWP",IF(D2="GG","XXGG","")))))
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{BE3C4938-8F19-4E3F-9C9A-34227C4C8923}" name="Beschreibung" dataDxfId="29">
+    <tableColumn id="27" xr3:uid="{BE3C4938-8F19-4E3F-9C9A-34227C4C8923}" name="Beschreibung" dataDxfId="40">
       <calculatedColumnFormula>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3309,8 +3309,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table3" displayName="Table3" ref="A1:E34">
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Wert"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Real" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Spiel" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Real" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Spiel" dataDxfId="38"/>
     <tableColumn id="5" xr3:uid="{16BD6806-29CB-4A81-B6F6-E74363828D03}" name="Skalierung real &gt; spiel"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Einheit"/>
   </tableColumns>
@@ -3343,19 +3343,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table6" displayName="Table6" ref="A1:L11">
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="WS"/>
-    <tableColumn id="12" xr3:uid="{EB8234D1-70DE-48AE-82B3-197397D4EA50}" name="HWB" dataDxfId="26"/>
-    <tableColumn id="7" xr3:uid="{382715DF-E649-4C68-8229-17F79CFD05E9}" name="Gas Real" dataDxfId="25"/>
-    <tableColumn id="8" xr3:uid="{9D3BFB1F-D194-4CFF-801A-646B03B69223}" name="Biomasse Real" dataDxfId="24"/>
-    <tableColumn id="9" xr3:uid="{92D64809-6003-4492-A647-B5959B9DDB64}" name="Fernwärme Real" dataDxfId="23"/>
-    <tableColumn id="10" xr3:uid="{08723E33-0A65-4BFC-9E7A-BA30B56D6C93}" name="Grünes Gas Real" dataDxfId="22"/>
-    <tableColumn id="11" xr3:uid="{308CC45B-DB70-43B9-B4BC-DFAA9033E01B}" name="Wärmepumpe Real" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Gas" dataDxfId="20">
+    <tableColumn id="12" xr3:uid="{EB8234D1-70DE-48AE-82B3-197397D4EA50}" name="HWB" dataDxfId="37"/>
+    <tableColumn id="7" xr3:uid="{382715DF-E649-4C68-8229-17F79CFD05E9}" name="Gas Real" dataDxfId="36"/>
+    <tableColumn id="8" xr3:uid="{9D3BFB1F-D194-4CFF-801A-646B03B69223}" name="Biomasse Real" dataDxfId="35"/>
+    <tableColumn id="9" xr3:uid="{92D64809-6003-4492-A647-B5959B9DDB64}" name="Fernwärme Real" dataDxfId="34"/>
+    <tableColumn id="10" xr3:uid="{08723E33-0A65-4BFC-9E7A-BA30B56D6C93}" name="Grünes Gas Real" dataDxfId="33"/>
+    <tableColumn id="11" xr3:uid="{308CC45B-DB70-43B9-B4BC-DFAA9033E01B}" name="Wärmepumpe Real" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Gas" dataDxfId="31">
       <calculatedColumnFormula>Table6[[#This Row],[Gas Real]]*years_per_round</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Biomasse">
       <calculatedColumnFormula>Table6[[#This Row],[Biomasse Real]]*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Fernwärme" dataDxfId="19">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Fernwärme" dataDxfId="30">
       <calculatedColumnFormula>Table6[[#This Row],[Fernwärme Real]]*years_per_round</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Grünes Gas">
@@ -3373,35 +3373,35 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table6_2" displayName="Table6_2" ref="A1:L11">
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="WS"/>
-    <tableColumn id="12" xr3:uid="{0F5289D2-6D79-4CC0-B64B-353B2E52E442}" name="HWB" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{7EE7A865-A9C3-4293-93B4-6A7F6B0D0739}" name="Gas Real" dataDxfId="17">
+    <tableColumn id="12" xr3:uid="{0F5289D2-6D79-4CC0-B64B-353B2E52E442}" name="HWB" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{7EE7A865-A9C3-4293-93B4-6A7F6B0D0739}" name="Gas Real" dataDxfId="28">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$23</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B9056603-4120-4751-8FD5-39C0A331CEB9}" name="Biomasse Real" dataDxfId="16">
+    <tableColumn id="8" xr3:uid="{B9056603-4120-4751-8FD5-39C0A331CEB9}" name="Biomasse Real" dataDxfId="27">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$24</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{775B0FD7-CE79-4EF3-8952-C905936C6A82}" name="Fernwärme Real" dataDxfId="15">
+    <tableColumn id="9" xr3:uid="{775B0FD7-CE79-4EF3-8952-C905936C6A82}" name="Fernwärme Real" dataDxfId="26">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$25</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{600AB853-60A0-47F9-B6B9-14F74CC0E0AE}" name="Grünes Gas Real" dataDxfId="14">
+    <tableColumn id="10" xr3:uid="{600AB853-60A0-47F9-B6B9-14F74CC0E0AE}" name="Grünes Gas Real" dataDxfId="25">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$26</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{1611B9F2-405C-4348-B6D7-02BE82C080AD}" name="Wärmepumpe Real" dataDxfId="13">
+    <tableColumn id="11" xr3:uid="{1611B9F2-405C-4348-B6D7-02BE82C080AD}" name="Wärmepumpe Real" dataDxfId="24">
       <calculatedColumnFormula>0</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Gas" dataDxfId="12">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Gas" dataDxfId="23">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Gas Real]]*'Mapping RealwerteSpielwerte'!$C$23+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Biomasse" dataDxfId="11">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Biomasse" dataDxfId="22">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Biomasse Real]]*'Mapping RealwerteSpielwerte'!$C$24+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Fernwärme" dataDxfId="10">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Fernwärme" dataDxfId="21">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Fernwärme Real]]*'Mapping RealwerteSpielwerte'!$C$25+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Grünes Gas" dataDxfId="9">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Grünes Gas" dataDxfId="20">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Grünes Gas Real]]*'Mapping RealwerteSpielwerte'!$C$26+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Wärmepumpe" dataDxfId="8">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Wärmepumpe" dataDxfId="19">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Wärmepumpe Real]]*'Mapping RealwerteSpielwerte'!$C$27+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3416,23 +3416,23 @@
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="WS"/>
-    <tableColumn id="8" xr3:uid="{9A60DCE1-E93F-4731-A39D-070BBC8CF024}" name="HWB" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{DB8D5F2F-7A4D-4517-BD90-EB468A9472F9}" name="Effizienz 0" dataDxfId="6">
+    <tableColumn id="8" xr3:uid="{9A60DCE1-E93F-4731-A39D-070BBC8CF024}" name="HWB" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{DB8D5F2F-7A4D-4517-BD90-EB468A9472F9}" name="Effizienz 0" dataDxfId="17">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_0</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Effizienz 1" dataDxfId="5">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Effizienz 1" dataDxfId="16">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Effizienz 2" dataDxfId="4">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Effizienz 2" dataDxfId="15">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Effizienz 3" dataDxfId="3">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Effizienz 3" dataDxfId="14">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Effizienz 4" dataDxfId="2">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Effizienz 4" dataDxfId="13">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Effizienz 5" dataDxfId="1">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Effizienz 5" dataDxfId="12">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_5</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3444,37 +3444,37 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Table8" displayName="Table8" ref="A1:L37">
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Netzbezug"/>
-    <tableColumn id="7" xr3:uid="{FA3BADB2-767D-406F-AE0E-3FD85C94E47C}" name="Netzbezug Real" dataDxfId="47">
+    <tableColumn id="7" xr3:uid="{FA3BADB2-767D-406F-AE0E-3FD85C94E47C}" name="Netzbezug Real" dataDxfId="11">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug]]*real_zu_spiel_netzbezug</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{7CF654A3-746E-45BB-8FE8-D85A1A2F26B3}" name="Kosten Real" dataDxfId="46">
+    <tableColumn id="12" xr3:uid="{7CF654A3-746E-45BB-8FE8-D85A1A2F26B3}" name="Kosten Real" dataDxfId="10">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*'Mapping RealwerteSpielwerte'!$B$27</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Budget" dataDxfId="45">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Budget" dataDxfId="9">
       <calculatedColumnFormula>-Table8[[#This Row],[Kosten Real]]*'Mapping RealwerteSpielwerte'!$C$27</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{CF2B80D5-564A-4F28-96D5-E05D40FB1362}" name="Emissionen Runde 1 Real" dataDxfId="44">
+    <tableColumn id="8" xr3:uid="{CF2B80D5-564A-4F28-96D5-E05D40FB1362}" name="Emissionen Runde 1 Real" dataDxfId="8">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{DDA1FEAD-C691-4D07-9868-BA59E3083198}" name="Emissionen Runde 2 Real" dataDxfId="43">
+    <tableColumn id="9" xr3:uid="{DDA1FEAD-C691-4D07-9868-BA59E3083198}" name="Emissionen Runde 2 Real" dataDxfId="7">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{FA64A352-3640-4484-B5E7-A06D893CF066}" name="Emissionen Runde 3 Real" dataDxfId="42">
+    <tableColumn id="10" xr3:uid="{FA64A352-3640-4484-B5E7-A06D893CF066}" name="Emissionen Runde 3 Real" dataDxfId="6">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D2D0C651-2DB4-4AE8-8AC2-5459168B14AC}" name="Emissionen Runde 4 Real" dataDxfId="41">
+    <tableColumn id="11" xr3:uid="{D2D0C651-2DB4-4AE8-8AC2-5459168B14AC}" name="Emissionen Runde 4 Real" dataDxfId="5">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="SP Runde 1" dataDxfId="40">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="SP Runde 1" dataDxfId="4">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="SP Runde 2" dataDxfId="39">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="SP Runde 2" dataDxfId="3">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="SP Runde 3" dataDxfId="38">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="SP Runde 3" dataDxfId="2">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="SP Runde 4" dataDxfId="37">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="SP Runde 4" dataDxfId="1">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3740,7 +3740,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:AA1000"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.453125" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -7839,7 +7839,7 @@
       <c r="X66" s="54"/>
       <c r="Y66" s="54"/>
       <c r="Z66" t="str">
-        <f t="shared" ref="Z66:Z100" si="2">_xlfn.TEXTJOIN(
+        <f t="shared" ref="Z66:Z72" si="2">_xlfn.TEXTJOIN(
 "XX",
 TRUE,
 IF(OR(F66="",F66=0),"",REPT(IF(F66&gt;0,"EN","EM"),ABS(F66))),
@@ -33311,7 +33311,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:V993"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.453125" customWidth="1"/>
     <col min="2" max="4" width="35.1796875" customWidth="1"/>
@@ -57990,7 +57990,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.54296875" customWidth="1"/>
     <col min="5" max="5" width="21.7265625" customWidth="1"/>
@@ -58559,7 +58559,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.54296875" customWidth="1"/>
     <col min="2" max="2" width="17.26953125" customWidth="1"/>
@@ -58654,40 +58654,40 @@
         <v>7</v>
       </c>
       <c r="B3" s="105">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C3" s="110" t="s">
         <v>277</v>
       </c>
       <c r="D3" s="105">
+        <v>0</v>
+      </c>
+      <c r="E3" s="105">
+        <v>1</v>
+      </c>
+      <c r="F3" s="105">
+        <v>2</v>
+      </c>
+      <c r="G3" s="105">
+        <v>3</v>
+      </c>
+      <c r="H3" s="105">
+        <v>4</v>
+      </c>
+      <c r="I3" s="105">
+        <v>5</v>
+      </c>
+      <c r="J3" s="105">
+        <v>6</v>
+      </c>
+      <c r="K3" s="105">
+        <v>7</v>
+      </c>
+      <c r="L3" s="105">
+        <v>8</v>
+      </c>
+      <c r="M3" s="105">
         <v>9</v>
-      </c>
-      <c r="E3" s="105">
-        <v>8</v>
-      </c>
-      <c r="F3" s="105">
-        <v>7</v>
-      </c>
-      <c r="G3" s="105">
-        <v>6</v>
-      </c>
-      <c r="H3" s="105">
-        <v>5</v>
-      </c>
-      <c r="I3" s="105">
-        <v>4</v>
-      </c>
-      <c r="J3" s="105">
-        <v>3</v>
-      </c>
-      <c r="K3" s="105">
-        <v>2</v>
-      </c>
-      <c r="L3" s="105">
-        <v>1</v>
-      </c>
-      <c r="M3" s="105">
-        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -58827,7 +58827,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="12.81640625" customWidth="1"/>
     <col min="10" max="10" width="13.81640625" customWidth="1"/>
@@ -59324,7 +59324,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="12.81640625" customWidth="1"/>
     <col min="10" max="10" width="13.81640625" customWidth="1"/>
@@ -59895,7 +59895,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="8" width="13.1796875" customWidth="1"/>
   </cols>
@@ -60338,7 +60338,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:L37"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7265625" customWidth="1"/>
     <col min="10" max="13" width="14" customWidth="1"/>

</xml_diff>